<commit_message>
scrape + maj master
</commit_message>
<xml_diff>
--- a/exports/notaires/annuaire_notaires_loire.xlsx
+++ b/exports/notaires/annuaire_notaires_loire.xlsx
@@ -692,7 +692,7 @@
       </c>
       <c r="L2" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:12</t>
+          <t>2026-06-24 15:10:26</t>
         </is>
       </c>
     </row>
@@ -754,7 +754,7 @@
       </c>
       <c r="L3" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:14</t>
+          <t>2026-06-24 15:10:27</t>
         </is>
       </c>
     </row>
@@ -808,7 +808,7 @@
       </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:16</t>
+          <t>2026-06-24 15:10:28</t>
         </is>
       </c>
     </row>
@@ -870,7 +870,7 @@
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:18</t>
+          <t>2026-06-24 15:10:29</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:19</t>
+          <t>2026-06-24 15:10:30</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="L7" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:20</t>
+          <t>2026-06-24 15:10:31</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:22</t>
+          <t>2026-06-24 15:10:32</t>
         </is>
       </c>
     </row>
@@ -1118,7 +1118,7 @@
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:23</t>
+          <t>2026-06-24 15:10:33</t>
         </is>
       </c>
     </row>
@@ -1180,7 +1180,7 @@
       </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:25</t>
+          <t>2026-06-24 15:10:34</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1242,7 @@
       </c>
       <c r="L11" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:27</t>
+          <t>2026-06-24 15:10:35</t>
         </is>
       </c>
     </row>
@@ -1304,7 +1304,7 @@
       </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:29</t>
+          <t>2026-06-24 15:10:36</t>
         </is>
       </c>
     </row>
@@ -1366,7 +1366,7 @@
       </c>
       <c r="L13" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:31</t>
+          <t>2026-06-24 15:10:37</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1428,7 @@
       </c>
       <c r="L14" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:33</t>
+          <t>2026-06-24 15:10:37</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
       </c>
       <c r="L15" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:35</t>
+          <t>2026-06-24 15:10:38</t>
         </is>
       </c>
     </row>
@@ -1544,7 +1544,7 @@
       </c>
       <c r="L16" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:36</t>
+          <t>2026-06-24 15:10:39</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
       </c>
       <c r="L17" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:38</t>
+          <t>2026-06-24 15:10:39</t>
         </is>
       </c>
     </row>
@@ -1668,7 +1668,7 @@
       </c>
       <c r="L18" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:39</t>
+          <t>2026-06-24 15:10:40</t>
         </is>
       </c>
     </row>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="L19" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:41</t>
+          <t>2026-06-24 15:10:41</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
       </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:42</t>
+          <t>2026-06-24 15:10:42</t>
         </is>
       </c>
     </row>
@@ -1854,7 +1854,7 @@
       </c>
       <c r="L21" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:44</t>
+          <t>2026-06-24 15:10:43</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1916,7 @@
       </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:46</t>
+          <t>2026-06-24 15:10:44</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:48</t>
+          <t>2026-06-24 15:10:45</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:49</t>
+          <t>2026-06-24 15:10:46</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2102,7 @@
       </c>
       <c r="L25" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:51</t>
+          <t>2026-06-24 15:10:47</t>
         </is>
       </c>
     </row>
@@ -2164,7 +2164,7 @@
       </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:54:47</t>
+          <t>2026-06-24 15:09:37</t>
         </is>
       </c>
     </row>
@@ -2226,7 +2226,7 @@
       </c>
       <c r="L27" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:54:49</t>
+          <t>2026-06-24 15:09:38</t>
         </is>
       </c>
     </row>
@@ -2288,7 +2288,7 @@
       </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:54:51</t>
+          <t>2026-06-24 15:09:39</t>
         </is>
       </c>
     </row>
@@ -2350,7 +2350,7 @@
       </c>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:54:53</t>
+          <t>2026-06-24 15:09:40</t>
         </is>
       </c>
     </row>
@@ -2412,7 +2412,7 @@
       </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:54:54</t>
+          <t>2026-06-24 15:09:41</t>
         </is>
       </c>
     </row>
@@ -2474,7 +2474,7 @@
       </c>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:54:56</t>
+          <t>2026-06-24 15:09:42</t>
         </is>
       </c>
     </row>
@@ -2536,7 +2536,7 @@
       </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:54:58</t>
+          <t>2026-06-24 15:09:43</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2598,7 @@
       </c>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:00</t>
+          <t>2026-06-24 15:09:44</t>
         </is>
       </c>
     </row>
@@ -2660,7 +2660,7 @@
       </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:01</t>
+          <t>2026-06-24 15:09:45</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2722,7 @@
       </c>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:03</t>
+          <t>2026-06-24 15:09:47</t>
         </is>
       </c>
     </row>
@@ -2784,7 +2784,7 @@
       </c>
       <c r="L36" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:05</t>
+          <t>2026-06-24 15:09:48</t>
         </is>
       </c>
     </row>
@@ -2846,7 +2846,7 @@
       </c>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:07</t>
+          <t>2026-06-24 15:09:49</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="L38" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:08</t>
+          <t>2026-06-24 15:09:50</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:10</t>
+          <t>2026-06-24 15:09:51</t>
         </is>
       </c>
     </row>
@@ -3032,7 +3032,7 @@
       </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:12</t>
+          <t>2026-06-24 15:09:51</t>
         </is>
       </c>
     </row>
@@ -3094,7 +3094,7 @@
       </c>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:13</t>
+          <t>2026-06-24 15:09:52</t>
         </is>
       </c>
     </row>
@@ -3156,7 +3156,7 @@
       </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:15</t>
+          <t>2026-06-24 15:09:53</t>
         </is>
       </c>
     </row>
@@ -3218,7 +3218,7 @@
       </c>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:17</t>
+          <t>2026-06-24 15:09:54</t>
         </is>
       </c>
     </row>
@@ -3280,7 +3280,7 @@
       </c>
       <c r="L44" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:18</t>
+          <t>2026-06-24 15:09:56</t>
         </is>
       </c>
     </row>
@@ -3342,7 +3342,7 @@
       </c>
       <c r="L45" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:20</t>
+          <t>2026-06-24 15:09:56</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       </c>
       <c r="L46" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:23</t>
+          <t>2026-06-24 15:09:57</t>
         </is>
       </c>
     </row>
@@ -3466,7 +3466,7 @@
       </c>
       <c r="L47" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:24</t>
+          <t>2026-06-24 15:09:59</t>
         </is>
       </c>
     </row>
@@ -3528,7 +3528,7 @@
       </c>
       <c r="L48" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:26</t>
+          <t>2026-06-24 15:10:00</t>
         </is>
       </c>
     </row>
@@ -3590,7 +3590,7 @@
       </c>
       <c r="L49" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:28</t>
+          <t>2026-06-24 15:10:01</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3652,7 @@
       </c>
       <c r="L50" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:29</t>
+          <t>2026-06-24 15:10:02</t>
         </is>
       </c>
     </row>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="L51" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:31</t>
+          <t>2026-06-24 15:10:02</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3776,7 @@
       </c>
       <c r="L52" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:33</t>
+          <t>2026-06-24 15:10:03</t>
         </is>
       </c>
     </row>
@@ -3838,7 +3838,7 @@
       </c>
       <c r="L53" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:35</t>
+          <t>2026-06-24 15:10:05</t>
         </is>
       </c>
     </row>
@@ -3900,7 +3900,7 @@
       </c>
       <c r="L54" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:36</t>
+          <t>2026-06-24 15:10:06</t>
         </is>
       </c>
     </row>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="L55" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:37</t>
+          <t>2026-06-24 15:10:06</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4024,7 @@
       </c>
       <c r="L56" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:39</t>
+          <t>2026-06-24 15:10:07</t>
         </is>
       </c>
     </row>
@@ -4086,7 +4086,7 @@
       </c>
       <c r="L57" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:41</t>
+          <t>2026-06-24 15:10:09</t>
         </is>
       </c>
     </row>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="L58" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:43</t>
+          <t>2026-06-24 15:10:10</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="L59" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:45</t>
+          <t>2026-06-24 15:10:11</t>
         </is>
       </c>
     </row>
@@ -4272,7 +4272,7 @@
       </c>
       <c r="L60" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:47</t>
+          <t>2026-06-24 15:10:12</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="L61" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:48</t>
+          <t>2026-06-24 15:10:13</t>
         </is>
       </c>
     </row>
@@ -4396,7 +4396,7 @@
       </c>
       <c r="L62" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:50</t>
+          <t>2026-06-24 15:10:14</t>
         </is>
       </c>
     </row>
@@ -4458,7 +4458,7 @@
       </c>
       <c r="L63" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:52</t>
+          <t>2026-06-24 15:10:15</t>
         </is>
       </c>
     </row>
@@ -4520,7 +4520,7 @@
       </c>
       <c r="L64" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:54</t>
+          <t>2026-06-24 15:10:16</t>
         </is>
       </c>
     </row>
@@ -4582,7 +4582,7 @@
       </c>
       <c r="L65" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:56</t>
+          <t>2026-06-24 15:10:16</t>
         </is>
       </c>
     </row>
@@ -4644,7 +4644,7 @@
       </c>
       <c r="L66" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:57</t>
+          <t>2026-06-24 15:10:18</t>
         </is>
       </c>
     </row>
@@ -4706,7 +4706,7 @@
       </c>
       <c r="L67" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:55:58</t>
+          <t>2026-06-24 15:10:18</t>
         </is>
       </c>
     </row>
@@ -4768,7 +4768,7 @@
       </c>
       <c r="L68" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:00</t>
+          <t>2026-06-24 15:10:19</t>
         </is>
       </c>
     </row>
@@ -4830,7 +4830,7 @@
       </c>
       <c r="L69" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:02</t>
+          <t>2026-06-24 15:10:20</t>
         </is>
       </c>
     </row>
@@ -4892,7 +4892,7 @@
       </c>
       <c r="L70" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:04</t>
+          <t>2026-06-24 15:10:21</t>
         </is>
       </c>
     </row>
@@ -4954,7 +4954,7 @@
       </c>
       <c r="L71" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:06</t>
+          <t>2026-06-24 15:10:21</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5016,7 @@
       </c>
       <c r="L72" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:07</t>
+          <t>2026-06-24 15:10:23</t>
         </is>
       </c>
     </row>
@@ -5078,7 +5078,7 @@
       </c>
       <c r="L73" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:08</t>
+          <t>2026-06-24 15:10:24</t>
         </is>
       </c>
     </row>
@@ -5132,7 +5132,7 @@
       </c>
       <c r="L74" s="5" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:10</t>
+          <t>2026-06-24 15:10:25</t>
         </is>
       </c>
     </row>
@@ -5194,7 +5194,7 @@
       </c>
       <c r="L75" s="7" t="inlineStr">
         <is>
-          <t>2026-06-24 14:56:11</t>
+          <t>2026-06-24 15:10:26</t>
         </is>
       </c>
     </row>

</xml_diff>